<commit_message>
Change sender name from Oseni Ibrahim to Victor Nweze everywhere
Rebuilt the invoice and German real estate workbooks; removed the now-redundant
older Victor Nweze invoice file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XwQBoB1SBrvgpAdZTTqNbP
</commit_message>
<xml_diff>
--- a/Germany_Real_Estate_Social_Media_Prospects_200.xlsx
+++ b/Germany_Real_Estate_Social_Media_Prospects_200.xlsx
@@ -798,7 +798,7 @@
 Beispiel: Wird in einem Ihrer Projekte eine Einheit verkauft, entsteht automatisch ein Update-Entwurf für Instagram und LinkedIn.
 Wäre das für Sie einen Blick wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -942,7 +942,7 @@
 So könnte etwa jede neue Villa automatisch einen hochwertigen Karussell-Entwurf erhalten, während Mietwohnungen kürzere Story-Texte bekommen.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1082,7 +1082,7 @@
 So könnte ein neues Gewerbeobjekt in Karlsruhe ohne zusätzlichen Aufwand als LinkedIn- und Facebook-Entwurf vorliegen.
 Soll ich Ihnen zeigen, wie das konkret aussieht?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1226,7 +1226,7 @@
 Eine neue Wohnung in Mannheim würde so automatisch als Feed-Post und Facebook-Beitrag vorbereitet, zur Freigabe durch Sie.
 Hätten Sie Lust auf ein kurzes Gespräch dazu?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1366,7 +1366,7 @@
 Beispiel: Das neue Mehrfamilienhaus in Stuttgart erscheint auf der Website, und kurz darauf liegt ein Instagram- und Facebook-Entwurf zur Freigabe bereit.
 Wäre das für Ihr Team interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1506,7 +1506,7 @@
 Etwa: Eine neue Mietwohnung auf Ihrer Mieten-Seite erzeugt sofort einen fertigen Story- und Feed-Entwurf.
 Hätten Sie Interesse, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1650,7 +1650,7 @@
 Konkret: Wird eine Wohnung in Degerloch als vermietet markiert, entsteht automatisch ein kurzer Facebook-Post dazu.
 Darf ich Ihnen das kurz an einem Beispiel zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1794,7 +1794,7 @@
 Ein neues Objekt auf Ihrer Objektseite würde so automatisch als Instagram- und Facebook-Entwurf vorliegen.
 Darf ich Ihnen das an einem Ihrer aktuellen Objekte skizzieren?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -1936,7 +1936,7 @@
 Beispiel: Meldet Ihr Vertrieb in Renningen eine Wohnung als reserviert, liegt kurz danach ein passender Post-Entwurf mit Projektbild zur Freigabe bereit.
 Wäre so ein Ablauf für Ihre Projekte grundsätzlich interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2074,7 +2074,7 @@
 Ein Beispiel: Wird im System ein neuer Bauabschnitt freigegeben, entsteht daraus automatisch ein Entwurf, den Ihr Team nur noch prüft.
 Darf ich Ihnen zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2222,7 +2222,7 @@
 Beispiel: Ein neues Video-Exposé auf YouTube löst automatisch einen passenden Instagram- und Facebook-Entwurf mit Link aus.
 Würde Sie ein kurzes Gespräch dazu interessieren?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2366,7 +2366,7 @@
 Beispiel: Ein neu angelegtes Haus erzeugt automatisch passende Entwürfe für Instagram und Facebook.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2500,7 +2500,7 @@
 So könnte etwa jedes neue Objekt am Ammersee automatisch einen Entwurf mit Standort-Hashtags für Herrsching erhalten.
 Wäre so etwas für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2644,7 +2644,7 @@
 Denkbar wäre etwa ein automatischer Entwurf pro Standort, sobald dort eine Etagenwohnung neu eingestellt wird.
 Wäre das einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2788,7 +2788,7 @@
 Konkret: Ist ein neuer Rundgang online, liegt ein Instagram-Entwurf mit Link zur 3D-Besichtigung für @immopartner.de bereit.
 Hätten Sie Lust, das kurz zu besprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -2932,7 +2932,7 @@
 Beispiel: Sobald eine Ihrer Wohnungen als vermietet markiert ist, liegt automatisch ein passender Instagram-Entwurf zur Freigabe bereit.
 Wäre das für Ihr Büro grundsätzlich interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3072,7 +3072,7 @@
 Konkret: Neues Objekt in Landshut online, und für @rathay_immobilien liegt direkt ein Karussell-Entwurf mit Kurztext bereit.
 Darf ich Ihnen zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3212,7 +3212,7 @@
 Ein Beispiel: Wird eine Ihrer Wohnungen reserviert, entsteht automatisch ein kurzer „Reserviert“-Post im Stil Ihres Accounts.
 Hätten Sie Interesse, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3355,7 +3355,7 @@
 Konkret könnte eine neu vermietete Wohnung in Wilmersdorf automatisch als 'Vermietet'-Post zur Freigabe bei Ihnen oder Herrn Bethke landen.
 Hätten Sie Lust, das einmal durchzusprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3494,7 +3494,7 @@
 Beispiel: Eine Kapitalanlage-Wohnung in Charlottenburg wird eingestellt, und Entwürfe für Instagram, Facebook und LinkedIn liegen parallel bereit.
 Wäre ein kurzer Austausch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3640,7 +3640,7 @@
 Konkret: Sie laden ein neues Objektvideo hoch, und für YouTube, Instagram und Facebook liegen passende Textentwürfe zur Freigabe bereit.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3782,7 +3782,7 @@
 Ein verkauftes Haus in Osterholz-Scharmbeck würde so direkt einen „Verkauft“-Entwurf auslösen.
 Hätten Sie Lust, das kurz zu besprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -3924,7 +3924,7 @@
 Beispiel: Sobald ein Haus in Bremerhaven online geht, liegt ein Post-Entwurf mit Link zum neuen Objektvideo bereit. Ihre kreativen Formate bleiben bei Ihnen.
 Wollen wir kurz darüber sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4066,7 +4066,7 @@
 Beispielsweise könnte eine Kapitalanlage automatisch einen sachlichen LinkedIn-Text erhalten, während dieselbe Wohnung für Instagram emotionaler formuliert wird.
 Wäre ein kurzes Gespräch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4210,7 +4210,7 @@
 So könnte ein als verkauft markiertes Haus direkt einen „Verkauft“-Post-Entwurf auslösen, den Sie nur noch freigeben.
 Wollen wir uns dazu kurz austauschen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4354,7 +4354,7 @@
 Beispiel: Eine neue Mietwohnung in Bornheim wird eingestellt, und kurz darauf liegt ein passender Instagram-Entwurf mit Stadtteil-Hashtags zur Freigabe bereit.
 Wäre das für Ihr Team interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4498,7 +4498,7 @@
 Konkret: Ein neues Einfamilienhaus in Göttingen erhält automatisch einen Post-Entwurf mit Göttinger Hashtags, ein Objekt in Kassel entsprechend eigene.
 Hätten Sie Lust auf einen kurzen Austausch dazu?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4642,7 +4642,7 @@
 Konkret könnte jedes neue Objekt einen Entwurf mit standortpassenden Hashtags (#wiesbaden, #mainz …) erhalten, und bei „verkauft“ entsteht automatisch ein Referenz-Post.
 Darf ich Ihnen zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4785,7 +4785,7 @@
 Eine neue Ferienwohnung mit Meerblick in Sellin könnte so direkt als Instagram- und Facebook-Entwurf vorliegen.
 Hätten Sie Interesse, darüber zu sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -4928,7 +4928,7 @@
 Ein Beispiel: Sie stellen eine Eigentumswohnung in Warnemünde ein, und der Beitragsentwurf für @drenkhahnimmobilien liegt direkt zur Prüfung bereit.
 Sollen wir uns dazu kurz austauschen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5071,7 +5071,7 @@
 So würde etwa aus einer Preisanpassung für ein Haus in Gehlsdorf automatisch ein kurzer Update-Beitrag, den Sie nur freigeben.
 Wäre das eine Entlastung für Ihr Team?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5210,7 +5210,7 @@
 Ein neues Objekt aus Ihrem Bestand könnte so ohne zusätzlichen Schreibaufwand als Beitrag für @engfer_und_partner_immo vorbereitet werden.
 Wollen wir darüber kurz sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5353,7 +5353,7 @@
 Konkret: Sobald ein Objekt in Schwerin als verkauft markiert ist, liegt der passende Beitrag für @die_immobilienexperten und Ihre Facebook-Seite bereit.
 Wäre das für IMMO-KONZEPTE interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5492,7 +5492,7 @@
 So würde eine neue Wohnung am Pfaffenteich automatisch als 'NEU'-Beitrag im gewohnten Stil zur Freigabe erscheinen.
 Wäre das eine Überlegung wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5632,7 +5632,7 @@
 Für Ihre Neubau-Vermarktung könnte zum Beispiel jede freigegebene Einheit automatisch einen eigenen Entwurf samt Grundriss-Hinweis erhalten.
 Wäre das eine sinnvolle Entlastung für Ihr Team?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5772,7 +5772,7 @@
 Eine neue Eigentumswohnung könnte so direkt als Instagram-Entwurf mit Eckdaten bereitstehen.
 Wäre das eine Überlegung für Ihr Haus wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -5916,7 +5916,7 @@
 Konkret: Sobald ein Objekt auf „verkauft“ gesetzt wird, liegt ein passender Entwurf für @degen_immobilien_dortmund zur Freigabe bereit.
 Hätten Sie Interesse, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6056,7 +6056,7 @@
 Beispiel: Eine neu eingestellte Wohnung erscheint automatisch als Entwurf für @immobilien.wiegand, inklusive Eckdaten und Bildauswahl.
 Wäre das für Ihr Team interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6198,7 +6198,7 @@
 Beispiel: Wird ein Mehrfamilienhaus in Leipzig als vermittelt markiert, entsteht ein diskreter „Erfolgreich vermittelt“-Entwurf ohne sensible Details.
 Wäre das für Ihr Team interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6342,7 +6342,7 @@
 Zum Beispiel wird eine neue Altbauwohnung in der Oberstadt sofort als Instagram- und Facebook-Entwurf vorbereitet.
 Darf ich Ihnen zeigen, wie das konkret aussieht?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6486,7 +6486,7 @@
 Ein Beispiel: Jede neue Vermietung in Mainz-Gonsenheim erzeugt automatisch einen Story- und einen Feed-Entwurf.
 Wäre ein kurzes Gespräch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6630,7 +6630,7 @@
 So könnte etwa jedes neue Objekt auf Ihrer Seite 'Häuser zum Kauf' sofort als Karussell-Entwurf für Instagram vorliegen.
 Wäre ein kurzer Austausch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6772,7 +6772,7 @@
 Zum Beispiel könnte jede Woche automatisch ein Entwurf „Neu zur Miete in Leipzig“ mit den drei jüngsten Wohnungen entstehen, den Ihr Team nur noch freigibt.
 Hätten Sie Interesse, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -6912,7 +6912,7 @@
 Sobald ein Objekt auf Ihrer Seite 'Immobilienangebote' erscheint, hätten Sie so automatisch einen Instagram- und Facebook-Entwurf vorliegen.
 Hätten Sie Interesse, sich das kurz anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7052,7 +7052,7 @@
 Eine neue Wohnung in Leipzig ginge dann automatisch als Entwurf an @immohal_leipzig, eine in Halle an @immohal_halle.
 Wollen wir kurz darüber sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7196,7 +7196,7 @@
 Wird etwa das Haus in Plötzky reserviert, läge automatisch ein passender Statusbeitrag zur Freigabe bereit.
 Wäre das eine Überlegung wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7334,7 +7334,7 @@
 Beispiel: Eine neu eingestellte 3-Zimmer-Wohnung in Kiel erscheint als Entwurf zur Freigabe, nach der Vermietung folgt automatisch ein „vermietet“-Hinweis.
 Wäre so etwas für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7472,7 +7472,7 @@
 Konkret: Ein neues Wohn- und Geschäftshaus im Exposé ergibt direkt einen fertigen Beitragsentwurf, den Ihr Team nur noch prüft und freigibt.
 Wäre das ein Thema, über das wir kurz sprechen könnten?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7614,7 +7614,7 @@
 Ein Beispiel: Ein neues Ferienhaus an der Lübecker Bucht wird im System angelegt, und Ihr Marketing erhält sofort einen fertigen Entwurf für Feed und Story zur Freigabe.
 Darf ich Ihnen kurz zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7752,7 +7752,7 @@
 Beispiel: Ein neues Haus wird angelegt, und ein Reel-Text samt Hashtags liegt bereit.
 Hätten Sie Interesse an einem kurzen Austausch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -7888,7 +7888,7 @@
 Ein Beispiel: Wird im Neubauprojekt eine Wohnung verkauft, entsteht automatisch ein 'Nur noch X Einheiten frei'-Entwurf.
 Wäre das für Sie einen Blick wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8032,7 +8032,7 @@
 Eine neue Mietwohnung würde dann in einem Schritt zum Instagram-Post, Facebook-Beitrag und Newsletter-Baustein.
 Darf ich Ihnen zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8176,7 +8176,7 @@
 So würde jede neue Anzeige unter 'Haus kaufen' automatisch zu einem Instagram-Entwurf.
 Hätten Sie Interesse an einem kurzen Gespräch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8312,7 +8312,7 @@
 Zum Beispiel: Ein neues Gewerbeobjekt erzeugt einen sachlichen LinkedIn-Entwurf, eine Mietwohnung dagegen einen Instagram-Post im gewohnten Stil.
 Wäre ein kurzer Austausch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8450,7 +8450,7 @@
 Nimmt Ihr Team eine neue Penthousewohnung auf, wartet ein Karussell-Entwurf mit Eckdaten zur Freigabe.
 Wäre es für Sie interessant, darüber kurz zu sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8590,7 +8590,7 @@
 Ein Beispiel: Eine neue Eigentumswohnung in Dresden-Plauen erzeugt gleichzeitig einen Instagram-Post, einen LinkedIn-Text für Kapitalanleger und einen Facebook-Beitrag.
 Hätten Sie Interesse an einem kurzen Austausch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8730,7 +8730,7 @@
 Konkret könnte jede neu eingestellte Wohnung in Magdeburg am selben Tag als Facebook-Entwurf bereitliegen.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -8874,7 +8874,7 @@
 Ein Beispiel: Jedes neue Angebot auf Ihrer Website erscheint als fertiger Instagram-Entwurf, den Sie nur noch freigeben.
 Wollen wir uns kurz dazu austauschen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9013,7 +9013,7 @@
 So könnte eine neue Eigentumswohnung im Kiez gleichzeitig als Entwurf für Facebook und Instagram vorliegen, ohne dass Sie etwas doppelt schreiben.
 Wäre das für Sie einen Blick wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9156,7 +9156,7 @@
 Konkret: Ein Haus in Groß Glienicke geht online, und Sie erhalten passende Vorschläge für Instagram und Facebook, die Sie nur noch freigeben.
 Hätten Sie Interesse, sich das kurz anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9299,7 +9299,7 @@
 Beispiel: Eine neue Wohnung in Babelsberg erscheint auf Ihrer Website, und kurz darauf liegt ein Beitragsentwurf mit Bildern und Eckdaten zur Freigabe bereit.
 Wäre das für Ihr Büro interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9441,7 +9441,7 @@
 So würde aus einem neu aufgenommenen Einfamilienhaus automatisch ein Entwurf entstehen, den Sie nur noch freigeben.
 Wäre das für Sie einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9585,7 +9585,7 @@
 Beispiel: Ein neues Anlageobjekt ergibt parallel einen LinkedIn-Entwurf mit Kennzahlen und einen Instagram-Post mit Bildern.
 Wäre das einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9729,7 +9729,7 @@
 Ein Beispiel: Bei einem neuen Objekt wird aus Exposé-Text und Fotos automatisch ein eleganter Karussell-Entwurf vorbereitet.
 Hätten Sie Interesse an einem kurzen Gespräch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -9868,7 +9868,7 @@
 Ein neues Ferienhaus bei Bergen würde dann direkt als Entwurf für Facebook und Instagram bereitstehen.
 Darf ich Ihnen das an einem Beispiel zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10007,7 +10007,7 @@
 Wenn Sie beispielsweise ein Grundstück in Bad Doberan einstellen, wartet kurz danach ein fertiger Post-Entwurf auf Ihre Freigabe.
 Klingt das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10147,7 +10147,7 @@
 Für ein Anlageobjekt wie das in der City könnte so ein LinkedIn-Post mit Rendite und Eckdaten entstehen, für Wohnungen eher ein Instagram-Karussell.
 Wäre ein kurzer Austausch dazu für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10285,7 +10285,7 @@
 Ein Beispiel für @bkwimmo: Jede neue Wohnung ergibt automatisch einen Entwurf mit den wichtigsten Eckdaten und dem Titelbild.
 Wäre das einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10425,7 +10425,7 @@
 Konkret: Sobald ein neues Haus auf Ihrer Seite 'Häuser Leipzig' erscheint, liegt automatisch ein Beitragsentwurf für Instagram bereit.
 Wäre das für Ihr Team interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10567,7 +10567,7 @@
 Konkret: Wird eine neue Eigentumswohnung online gestellt, liegt parallel ein Entwurf für alle drei Kanäle zur Prüfung bereit.
 Wäre es sinnvoll, darüber einmal kurz zu sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10703,7 +10703,7 @@
 Ein neues Angebot auf Ihrer Seite „Alle Immobilien“ würde so direkt als Post-Entwurf zur Freigabe bereitstehen.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10839,7 +10839,7 @@
 Zum Beispiel: Ein neues Mehrfamilienhaus erzeugt automatisch einen sachlichen LinkedIn-Entwurf für Kapitalanleger und parallel einen Instagram-Post.
 Wäre das für Sie ein Thema?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -10975,7 +10975,7 @@
 Beispiel: Wandert ein Haus in Durlach ins Verkauft-Archiv, liegt automatisch ein passender Post bereit.
 Wäre das einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11111,7 +11111,7 @@
 Ein „Verkauft“-Status würde dann direkt einen sachlichen LinkedIn-Entwurf auslösen.
 Wäre ein kurzer Austausch für Sie und Herrn Kiefer interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11247,7 +11247,7 @@
 Konkret: Jede neu eingestellte Mietwohnung würde parallel als Facebook-Entwurf bereitstehen, den Sie nur noch freigeben.
 Wäre das grundsätzlich ein Thema für Sie?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11381,7 +11381,7 @@
 Konkret: Wird eine Mietwohnung in Neuenstadt eingestellt, liegt ein fertiger Beitragsentwurf bereit; ist sie vermietet, folgt ein kurzer „Vermietet“-Post zur Freigabe.
 Wäre das für Sie ein Thema, über das wir kurz sprechen könnten?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11517,7 +11517,7 @@
 Zum Beispiel ein automatischer Wochenpost „Neu zu vermieten in Augsburg“.
 Wäre das für Sie von Interesse?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11657,7 +11657,7 @@
 Ein Beispiel: Eine neue Wohnung, die Sie bei ImmoScout24 einstellen, erscheint kurz danach als Instagram-Entwurf in Ihrem Postfach.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11793,7 +11793,7 @@
 Etwa: Jede neue Eigentumswohnung im Portal ergibt automatisch einen Facebook-Entwurf zur Freigabe.
 Wäre das für Sie überlegenswert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -11937,7 +11937,7 @@
 Beispiel: Meldet ein Kollege ein Objekt als verkauft, entsteht automatisch ein „Erfolgreich vermittelt“-Beitrag zur Freigabe.
 Wäre das für Sie ein interessanter Gedanke?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12077,7 +12077,7 @@
 Zum Beispiel: Wird eine Loftfläche frei, entsteht direkt ein LinkedIn-Entwurf für Gewerbemieter.
 Wäre das für Sie einen Blick wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12209,7 +12209,7 @@
 Zum Beispiel ein wöchentlicher Sammelbeitrag „Neu in Regensburg“ und ein separater für München, beide automatisch vorbefüllt.
 Wäre ein kurzer Austausch dazu für Sie denkbar?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12353,7 +12353,7 @@
 Beispiel: Wird eine Wohnung in Kolbermoor als verkauft markiert, entsteht automatisch ein kurzer Dankes-Post.
 Wäre das eine Entlastung, über die wir kurz sprechen könnten?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12489,7 +12489,7 @@
 Beispiel: Sind in einem Neubauprojekt die letzten Einheiten reserviert, liegt automatisch ein LinkedIn-Entwurf dazu bereit.
 Darf ich Ihnen das kurz skizzieren?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12623,7 +12623,7 @@
 Beispiel: Eine neue Villa mit Bootshaus wird automatisch zum Karussell-Entwurf mit Seeblick-Fotos.
 Darf ich Ihnen das kurz vorstellen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12759,7 +12759,7 @@
 Für Sie denkbar: Jede neue Wohnung aus dem Portfolio erscheint als fertiger Facebook-Entwurf, auf Wunsch zusätzlich für Instagram.
 Wäre das ein Thema, über das wir kurz sprechen könnten?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -12890,7 +12890,7 @@
 So könnte etwa jede neue Mietwohnung in Potsdam-West automatisch als Beitragsvorschlag bei Ihnen landen.
 Darf ich Ihnen zeigen, wie das bei Ihnen aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13028,7 +13028,7 @@
 So könnte ein neues Objekt direkt einen LinkedIn-Entwurf und einen kurzen Facebook-Post erhalten.
 Darf ich Ihnen das einmal kurz skizzieren?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13162,7 +13162,7 @@
 So könnte etwa ein wöchentlicher Entwurf entstehen: „Noch drei Wohnungen im FLAIR verfügbar“, mit Grundrissbild zur Freigabe.
 Ist das ein Thema, das für Sie interessant sein könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13296,7 +13296,7 @@
 Ein Reihenhaus in Schnelsen, das Sie einstellen, würde so direkt als Entwurf für alle drei Kanäle vorliegen – Sie prüfen nur noch.
 Wäre das einen kurzen Austausch wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13432,7 +13432,7 @@
 Beispiel: Eine neue Wohnung wird eingestellt, und der passende Instagram-Entwurf ist wenige Minuten später bereit.
 Wollen wir kurz darüber sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13572,7 +13572,7 @@
 Eine neue Wohnung in Hausen könnte so ohne Mehrarbeit als Beitragsentwurf bereitstehen.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13708,7 +13708,7 @@
 Beispiel: Eine neu verfügbare Gewerbefläche wird automatisch zu einem sachlichen LinkedIn-Entwurf mit den wichtigsten Eckdaten.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13844,7 +13844,7 @@
 Ein Mietshaus in Hochheim könnte so ohne Mehraufwand als Facebook- und Instagram-Entwurf erscheinen.
 Darf ich Ihnen das kurz zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -13983,7 +13983,7 @@
 Beispiel: Eine Wohnung in Sassnitz wird eingestellt, und der passende Facebook-Beitrag steht kurz darauf zur Freigabe bereit.
 Wäre das für Ihr Familienunternehmen hilfreich?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14114,7 +14114,7 @@
 Zum Beispiel: Wird eine Altbauwohnung in der KTV vermietet, entsteht automatisch ein kurzer 'Vermietet'-Beitrag zur Freigabe.
 Wäre so etwas für Sie denkbar?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14249,7 +14249,7 @@
 Eine Ferienwohnung mit Seeblick in Bansin wäre so ohne zusätzlichen Schreibaufwand als Beitrag vorbereitet.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14387,7 +14387,7 @@
 Ein neues Objekt würde dann direkt als Beitragsentwurf vorliegen, den Sie nur noch kurz prüfen.
 Hätten Sie Interesse, das einmal durchzusprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14525,7 +14525,7 @@
 Eine neue Wohnung in Waldhausen könnte so ohne zusätzliches Schreiben als fertiger Entwurf in Ihrer Freigabe landen.
 Wäre das für Sie ein interessantes Thema?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14661,7 +14661,7 @@
 Eine neue Mietwohnung könnte so ohne zusätzlichen Aufwand als Instagram-Entwurf zur Freigabe bereitliegen.
 Hätten Sie Lust auf einen kurzen Austausch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14793,7 +14793,7 @@
 Eine neue Ankermieter-Vermietung in einem Fachmarktzentrum würde so direkt als LinkedIn-Entwurf zur Freigabe vorliegen.
 Wäre ein kurzes Gespräch dazu denkbar?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -14925,7 +14925,7 @@
 Die Parkresidenz Gut Ludenberg wäre dann zum Beispiel sofort als fertiger Post-Entwurf zur Freigabe vorhanden.
 Darf ich Ihnen das an einem Beispiel zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15061,7 +15061,7 @@
 Nach einem Closing läge etwa sofort ein anonymisierter LinkedIn-Entwurf mit Assetklasse, Lage und Rolle von rheinwert bereit.
 Wäre das für Sie ein interessanter Gedanke?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15201,7 +15201,7 @@
 So könnte ein verkauftes Mehrfamilienhaus direkt einen fertigen „Verkauft“-Post für Instagram und Facebook erzeugen, den Sie nur noch freigeben.
 Darf ich Ihnen kurz zeigen, wie das aussieht?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15339,7 +15339,7 @@
 Konkret könnte jeder Standort monatlich automatisch einen Entwurf „Neu im Angebot“ erhalten, im einheitlichen Hammers-&amp;-Heinz-Stil und von Ihnen nur noch freigegeben.
 Hätten Sie Interesse an einem kurzen Gespräch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15471,7 +15471,7 @@
 Aus einer neuen Wohnung würde so direkt ein Post-Entwurf, den Sie nur noch prüfen.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15615,7 +15615,7 @@
 Eine neue Wohnung würde so automatisch zum fertigen Facebook-Entwurf, den Sie nur noch freigeben.
 Wollen wir kurz darüber sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15755,7 +15755,7 @@
 Eine neue Wohnung in der Neustadt würde dann direkt als fertiger Entwurf in Ihrer Freigabeliste landen.
 Wäre das eine Überlegung wert?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -15895,7 +15895,7 @@
 So würde etwa eine neu eingestellte Wohnung in Chemnitz automatisch als Beitragsentwurf bei Ihnen landen.
 Hätten Sie Lust, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16027,7 +16027,7 @@
 Beispiel: Eine neue Villa wird automatisch zu einem Beitragsentwurf, den Sie nur noch freigeben.
 Sollen wir darüber kurz sprechen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16163,7 +16163,7 @@
 Beispiel: Wird ein Objekt als verkauft markiert, erhalten Sie direkt einen 'Erfolgreich vermittelt'-Beitrag zur Freigabe.
 Darf ich Ihnen das kurz zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16303,7 +16303,7 @@
 Eine neue Gewerbefläche in Magdeburg würde so direkt als LinkedIn-Entwurf vorliegen, eine Wohnung parallel als Facebook-Beitrag.
 Darf ich Ihnen ein kurzes Beispiel schicken?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16433,7 +16433,7 @@
 Eine frei werdende Wohnung ergäbe so automatisch einen fertigen Entwurf.
 Wäre das für Sie überhaupt ein Thema?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16571,7 +16571,7 @@
 Eine neue Altbauwohnung in St. Gertrud würde dann als Entwurf für Facebook und Instagram bereitliegen.
 Darf ich Ihnen das bei Gelegenheit kurz zeigen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16705,7 +16705,7 @@
 Ein neues Landhaus in Ostholstein ergäbe so direkt einen fertigen Entwurf zur Freigabe.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16841,7 +16841,7 @@
 Gerade Kapitalanlageobjekte ließen sich so automatisch als sachlicher LinkedIn-Beitrag für Investoren vorbereiten.
 Wäre das für Sie ein Thema?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -16977,7 +16977,7 @@
 Konkret: Eine frei werdende Wohnung in Gotha würde automatisch als Facebook-Entwurf mit Ortsbezug vorbereitet.
 Wäre das interessant für Sie?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -17703,7 +17703,7 @@
 Beispiel: Ein neues Einfamilienhaus in Waldkirch erscheint automatisch als abgestimmter Entwurf für Instagram und Facebook.
 Wer wäre bei Ihnen der richtige Ansprechpartner dafür?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -17839,7 +17839,7 @@
 So könnte etwa jede verkaufte Wohnung in Biebrich automatisch einen kurzen Referenz-Post vorbereiten.
 Wäre das für Sie ein Thema?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -17971,7 +17971,7 @@
 Eine neue Wohnung im Rheingauviertel läge dann ohne Zusatzaufwand als Post-Entwurf zur Freigabe bereit.
 Hätten Sie Interesse, sich das einmal anzusehen?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -18107,7 +18107,7 @@
 Ein Reihenhaus in Hechtsheim könnte so beispielsweise automatisch als Facebook-Beitrag mit passenden lokalen Hashtags vorbereitet werden.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -18239,7 +18239,7 @@
 Eine frei werdende Wohnung in der Gießener Nordstadt könnte so direkt als Entwurf bereitstehen, sobald sie im System angelegt ist.
 Darf ich Ihnen zeigen, wie das aussehen könnte?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -18371,7 +18371,7 @@
 Konkret: Eine neue Wohnung im Martinsviertel wird automatisch als Karussell-Entwurf mit den Exposé-Fotos vorbereitet.
 Wäre das für Sie interessant?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>
@@ -18507,7 +18507,7 @@
 Bei einer Jugendstilvilla auf der Mathildenhöhe entstünde so automatisch ein Entwurf, der Baujahr und Denkmalstatus aufgreift.
 Hätten Sie Interesse an einem kurzen Austausch?
 Mit freundlichen Grüßen
-Oseni Ibrahim
+Victor Nweze
 Real Estate Automation Specialist</t>
         </is>
       </c>

</xml_diff>